<commit_message>
Best time to sell and buy
</commit_message>
<xml_diff>
--- a/dsa-doc/dsa-problems.xlsx
+++ b/dsa-doc/dsa-problems.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shubh\Projects\DSA\dsa-doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E454DED3-5048-4353-8DD6-1CFBB8C51F3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83E164A6-16DA-4905-BA01-A04761764F29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="853" uniqueCount="555">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="858" uniqueCount="555">
   <si>
     <t>Num</t>
   </si>
@@ -2561,7 +2561,9 @@
       <c r="E15" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="F15" s="6"/>
+      <c r="F15" s="6" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="16" spans="1:6" ht="15" thickBot="1">
       <c r="A16" s="6">
@@ -5354,21 +5356,33 @@
       </c>
     </row>
     <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>325</v>
+      </c>
       <c r="B5" s="14" t="s">
         <v>332</v>
       </c>
     </row>
     <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>325</v>
+      </c>
       <c r="B6" s="14" t="s">
         <v>333</v>
       </c>
     </row>
     <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>325</v>
+      </c>
       <c r="B7" s="14" t="s">
         <v>334</v>
       </c>
     </row>
     <row r="8" spans="1:2">
+      <c r="A8" t="s">
+        <v>325</v>
+      </c>
       <c r="B8" s="14" t="s">
         <v>335</v>
       </c>
@@ -6506,6 +6520,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">

</xml_diff>

<commit_message>
contest problem and theory of Trees
</commit_message>
<xml_diff>
--- a/dsa-doc/dsa-problems.xlsx
+++ b/dsa-doc/dsa-problems.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shubh\Projects\DSA\dsa-doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83E164A6-16DA-4905-BA01-A04761764F29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CD19E76-7BD8-4600-8A86-0166D598A4AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,6 @@
     <sheet name="Sheet2" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -28,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="858" uniqueCount="555">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="895" uniqueCount="555">
   <si>
     <t>Num</t>
   </si>
@@ -2581,7 +2580,9 @@
       <c r="E16" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="F16" s="6"/>
+      <c r="F16" s="6" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="17" spans="1:6" ht="15" thickBot="1">
       <c r="A17" s="6">
@@ -2599,7 +2600,9 @@
       <c r="E17" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F17" s="6"/>
+      <c r="F17" s="6" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="18" spans="1:6" ht="15" thickBot="1">
       <c r="A18" s="6">
@@ -2617,7 +2620,9 @@
       <c r="E18" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F18" s="6"/>
+      <c r="F18" s="6" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="19" spans="1:6" ht="15" thickBot="1">
       <c r="A19" s="6">
@@ -2635,7 +2640,9 @@
       <c r="E19" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F19" s="6"/>
+      <c r="F19" s="6" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="20" spans="1:6" ht="15" thickBot="1">
       <c r="A20" s="9">
@@ -2653,7 +2660,9 @@
       <c r="E20" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="F20" s="9"/>
+      <c r="F20" s="9" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="21" spans="1:6" ht="15" thickBot="1">
       <c r="A21" s="9">
@@ -2671,7 +2680,9 @@
       <c r="E21" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="F21" s="9"/>
+      <c r="F21" s="9" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="22" spans="1:6" ht="15" thickBot="1">
       <c r="A22" s="4">
@@ -2689,7 +2700,9 @@
       <c r="E22" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="F22" s="4"/>
+      <c r="F22" s="4" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="23" spans="1:6" ht="15" thickBot="1">
       <c r="A23" s="6">
@@ -2707,7 +2720,9 @@
       <c r="E23" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F23" s="6"/>
+      <c r="F23" s="6" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="24" spans="1:6" ht="15" thickBot="1">
       <c r="A24" s="6">
@@ -2725,7 +2740,9 @@
       <c r="E24" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F24" s="6"/>
+      <c r="F24" s="6" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="25" spans="1:6" ht="15" thickBot="1">
       <c r="A25" s="6">
@@ -2743,7 +2760,9 @@
       <c r="E25" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F25" s="6"/>
+      <c r="F25" s="6" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="26" spans="1:6" ht="15" thickBot="1">
       <c r="A26" s="6">
@@ -2761,7 +2780,9 @@
       <c r="E26" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F26" s="6"/>
+      <c r="F26" s="6" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="27" spans="1:6" ht="15" thickBot="1">
       <c r="A27" s="6">
@@ -2779,7 +2800,9 @@
       <c r="E27" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F27" s="6"/>
+      <c r="F27" s="6" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="28" spans="1:6" ht="15" thickBot="1">
       <c r="A28" s="9">
@@ -2797,7 +2820,9 @@
       <c r="E28" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="F28" s="9"/>
+      <c r="F28" s="9" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="29" spans="1:6" ht="15" thickBot="1">
       <c r="A29" s="4">
@@ -2815,7 +2840,9 @@
       <c r="E29" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="F29" s="4"/>
+      <c r="F29" s="4" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="30" spans="1:6" ht="15" thickBot="1">
       <c r="A30" s="6">
@@ -2833,7 +2860,9 @@
       <c r="E30" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F30" s="6"/>
+      <c r="F30" s="6" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="31" spans="1:6" ht="15" thickBot="1">
       <c r="A31" s="6">
@@ -2851,7 +2880,9 @@
       <c r="E31" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F31" s="6"/>
+      <c r="F31" s="6" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="32" spans="1:6" ht="15" thickBot="1">
       <c r="A32" s="6">
@@ -2869,7 +2900,9 @@
       <c r="E32" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F32" s="6"/>
+      <c r="F32" s="6" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="33" spans="1:6" ht="15" thickBot="1">
       <c r="A33" s="6">
@@ -2887,7 +2920,9 @@
       <c r="E33" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F33" s="6"/>
+      <c r="F33" s="6" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="34" spans="1:6" ht="15" thickBot="1">
       <c r="A34" s="6">
@@ -2905,7 +2940,9 @@
       <c r="E34" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F34" s="6"/>
+      <c r="F34" s="6" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="35" spans="1:6" ht="15" thickBot="1">
       <c r="A35" s="9">
@@ -2923,7 +2960,9 @@
       <c r="E35" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="F35" s="9"/>
+      <c r="F35" s="9" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="36" spans="1:6" ht="15" thickBot="1">
       <c r="A36" s="4">
@@ -2941,7 +2980,9 @@
       <c r="E36" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="F36" s="4"/>
+      <c r="F36" s="4" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="37" spans="1:6" ht="15" thickBot="1">
       <c r="A37" s="4">
@@ -2959,7 +3000,9 @@
       <c r="E37" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="F37" s="4"/>
+      <c r="F37" s="4" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="38" spans="1:6" ht="15" thickBot="1">
       <c r="A38" s="6">
@@ -2977,7 +3020,9 @@
       <c r="E38" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F38" s="6"/>
+      <c r="F38" s="6" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="39" spans="1:6" ht="15" thickBot="1">
       <c r="A39" s="6">
@@ -2995,7 +3040,9 @@
       <c r="E39" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F39" s="6"/>
+      <c r="F39" s="6" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="40" spans="1:6" ht="15" thickBot="1">
       <c r="A40" s="6">
@@ -3013,7 +3060,9 @@
       <c r="E40" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F40" s="6"/>
+      <c r="F40" s="6" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="41" spans="1:6" ht="15" thickBot="1">
       <c r="A41" s="6">
@@ -3031,7 +3080,9 @@
       <c r="E41" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F41" s="6"/>
+      <c r="F41" s="6" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="42" spans="1:6" ht="15" thickBot="1">
       <c r="A42" s="4">
@@ -3049,7 +3100,9 @@
       <c r="E42" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="F42" s="4"/>
+      <c r="F42" s="4" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="43" spans="1:6" ht="15" thickBot="1">
       <c r="A43" s="6">
@@ -3067,7 +3120,9 @@
       <c r="E43" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F43" s="6"/>
+      <c r="F43" s="6" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="44" spans="1:6" ht="15" thickBot="1">
       <c r="A44" s="6">
@@ -3085,7 +3140,9 @@
       <c r="E44" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F44" s="6"/>
+      <c r="F44" s="6" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="45" spans="1:6" ht="15" thickBot="1">
       <c r="A45" s="9">
@@ -3103,7 +3160,9 @@
       <c r="E45" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="F45" s="9"/>
+      <c r="F45" s="9" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="46" spans="1:6" ht="15" thickBot="1">
       <c r="A46" s="9">
@@ -3121,7 +3180,9 @@
       <c r="E46" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="F46" s="9"/>
+      <c r="F46" s="9" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="47" spans="1:6" ht="15" thickBot="1">
       <c r="A47" s="4">
@@ -3139,7 +3200,9 @@
       <c r="E47" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="F47" s="4"/>
+      <c r="F47" s="4" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="48" spans="1:6" ht="15" thickBot="1">
       <c r="A48" s="4">
@@ -3157,7 +3220,9 @@
       <c r="E48" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="F48" s="4"/>
+      <c r="F48" s="4" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="49" spans="1:6" ht="15" thickBot="1">
       <c r="A49" s="4">
@@ -3175,7 +3240,9 @@
       <c r="E49" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="F49" s="4"/>
+      <c r="F49" s="4" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="50" spans="1:6" ht="15" thickBot="1">
       <c r="A50" s="4">
@@ -3193,7 +3260,9 @@
       <c r="E50" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="F50" s="4"/>
+      <c r="F50" s="4" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="51" spans="1:6" ht="15" thickBot="1">
       <c r="A51" s="4">
@@ -3211,7 +3280,9 @@
       <c r="E51" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="F51" s="4"/>
+      <c r="F51" s="4" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="52" spans="1:6" ht="15" thickBot="1">
       <c r="A52" s="4">
@@ -3229,7 +3300,9 @@
       <c r="E52" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="F52" s="4"/>
+      <c r="F52" s="4" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="53" spans="1:6" ht="15" thickBot="1">
       <c r="A53" s="6">

</xml_diff>